<commit_message>
post-audit fixes: RMSF-orthogonal residue attribution, equilibration discard, suitability screening, deterministic clustering
</commit_message>
<xml_diff>
--- a/validation/SciML-MD_Validation_Tracker.xlsx
+++ b/validation/SciML-MD_Validation_Tracker.xlsx
@@ -294,382 +294,382 @@
     <t xml:space="preserve">Pearson r = 1.0000000000 between published residue scores and raw RMSF (1VII)</t>
   </si>
   <si>
-    <t xml:space="preserve">Displacement-weighted anomaly participation blended with RMSF (PARTIAL - see E-1)</t>
+    <t xml:space="preserve">Superseded by scoring/residue_attribution.py - RMSF-orthogonal attribution (see E-1 resolution)</t>
   </si>
   <si>
     <t xml:space="preserve">test_residue_scores_not_pure_rmsf; validation/revalidation.py::R1</t>
   </si>
   <si>
+    <t xml:space="preserve">D-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residue keys collided across chains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key str(residue) e.g. 'MET41' is not unique in multi-chain proteins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8H0R: 182 residues -&gt; 91 dict entries; chain A silently overwritten by chain B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain-disambiguated keys (NAME###_chainK) when duplicates occur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_residue_keys_do_not_collide_across_chains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tools/export_for_asvs.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASVS export produced constant values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read column 'score' (pipeline writes 'score_dynamic'); looked up residues by index (file keyed by name)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exports/8H0R/anomaly_residue.json = 0.25 for all 182 residues x 100 frames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reads score_dynamic (/100); positional residue mapping; pipeline now writes residue_scores_rmsf.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_asvs_export_not_constant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">msm/validation.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chapman-Kolmogorov test compared mismatched state spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P(k*tau) matrices estimated on different active sets compared without remapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test invalid whenever any state pruned - i.e. in every run performed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation runner embeds each MSM into full label space before comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/layer2_msm_validity.py::run_ck (executed on 4 systems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">msm/select_lag_and_dim.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAMP-2 scorer numerically unstable on real features</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cholesky-inverse whitening with reg=1e-6 on ill-conditioned covariances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returned 2.5e5 where valid VAMP-2 &lt;= dim (5); correct on random data, which is why mock tests missed it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-scored with deeptime VAMP.score(r=2), 80/20 split; repo values retained for record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/layer2_msm_validity.py::run_vamp2 (executed on 3 systems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">run_all_proteins.py / batch_runner.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVATION: mean frame score ~50 is a normalisation artifact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank normalisation forces uniform [0,1] per signal; fused mean = 0.5 by construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Info</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured 47.4-50.9 across all systems regardless of protein or dynamics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not a defect - documented; must never be reported as a health metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documented in VALIDATION_REPORT.md 2.3 and 8.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">deeptime KMeans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVATION: clustering not reproducible across machines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">deeptime KMeans platform-dependent despite fixed seed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARI 0.43-0.51 vs reference artifacts; 90/100 frames relabelled; tICA reproduces at r=0.96-0.9996</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIXED: sklearn Lloyd KMeans + canonical relabelling by sorted cluster centres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_clustering_is_deterministic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sampling / trajectory length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSERVATION: 100-frame trajectories cannot support MSM validity claims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insufficient sampling: few transitions per state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CK intervals +/-0.3-0.5 (no power); ITS unconverged (1VII +50%); pi CI 1.1-1.6x the value; VAMP-2 saturates at dim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open - regenerate at 50,000-step protocol or use public long-trajectory dataset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/layer2_msm_validity.py (all four systems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: residue scores still ~99% collinear with RMSF after the D-04 fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displacement-weighted participation is near-constant across residues; RMSF term dominates variance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-fix Pearson r vs RMSF = 0.996 (1VII), 0.990 (8H0R), 0.992 (1UBQ) - was 1.000 pre-fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESOLVED: scoring/residue_attribution.py (KSD-RA + explicit RMSF orthogonalisation). Spearman vs RMSF now -0.012 / +0.016 / +0.021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_residue_attribution_is_orthogonal_to_rmsf; validation/postaudit_results.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/layer3_external.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: B-factor correlation is fully explained by RMSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dynamic score is ~99% RMSF (see E-1), so B-factor agreement carries no anomaly-specific signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial Spearman(B, score | RMSF) = -0.019 (8H0R), -0.181 (1UBQ) - anomaly component adds nothing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - cannot be cited as external validation of the method; validates RMSF only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/revalidation.py::R3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: rare-STATE baseline comparison is circular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labels defined from pi (bottom quartile); rarity channel IS 1-pi - detector and label are the same quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Without rarity: 8H0R 0.83 vs LOF 0.93 (LOSES); 1CRN 0.76 vs IsoForest 0.85 (LOSES); 1UBQ 0.69 vs 0.70 (TIES); wins only 1VII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - must not be presented as a benchmark win; needs MSM-independent ground truth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/revalidation.py::R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: rare-TRANSITION 'headline figure' also circular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">surprise = -log P; P row-normalised from the same count matrix that defines the labels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spearman(surprise, -transition count) = 0.69 (1UBQ), 0.87 (1CRN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - withdraw as headline benchmark claim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/revalidation.py::R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/layer2_msm_validity.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: VAMP-2 saturation attributed to overfitting; actually a degenerate test set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 frames -&gt; 20 test frames -&gt; only 5 lagged pairs at lag 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conclusion (cannot justify hyper-parameters) unchanged; stated mechanism was wrong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documented - re-run when trajectories are longer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/revalidation.py::R6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALIDATION_REPORT.md 3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERRATUM: edge-case count stated as 21; actual suite is 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prose written from an earlier draft of the suite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edge_results_POSTFIX.json contains 25 cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrected in ERRATA section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/revalidation.py::R7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default moving-median smoothing erases isolated single-frame anomalies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moving_median(window=3..5) is applied unconditionally to the fused score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 1 seeded-anomaly test: scattered-mode AUROC 0.839 unsmoothed vs 0.550 at window=3 (-0.29). The pipeline is blind to transient rare events at default settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smoothing now opt-in: window default 1 (OFF) in run_all_proteins + batch_runner; CSV also carries a reference score_dynamic_smoothed_w5 column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_smoothing_is_off_by_default; test_isolated_spike_survives_default_scoring; validation/d09_impact.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHASE 1: pipeline loses to a trivial baseline on seeded structural anomalies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">450 K frames are globally expanded; RMSD-from-mean separates them perfectly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst mode: rmsd_from_mean AUROC 1.000 vs pipeline_fused 0.831. Acceptance criterion A2 FAILED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - either restrict claims to kinetic anomalies, or demonstrate added value over RMSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/phase1_seeded_anomaly.py (5 replicates, pre-registered criteria)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHASE 1: transition surprise is BELOW chance on sustained rare states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within a contiguous rare-state block, hot-&gt;hot transitions are self-consistent so P is high and surprise LOW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst mode surprise_only AUROC 0.351 (below 0.5 = anti-correlated with truth)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - surprise detects state CHANGES, not sustained residence in a rare state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/phase1_seeded_anomaly.py burst mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHASE 2: kinetic channel detects geometrically invisible transitions (B1 marginally missed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temporal scrambling: real frames, identical ensemble, only frame ORDER altered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">near mode: surprise 0.741 +/- 0.113 vs frame_to_frame_rmsd 0.500 and all time-blind detectors 0.471-0.546. B1 missed by 0.009 (bar 0.75); B2 and B4 passed decisively</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN - replicate on longer trajectories (ATLAS/mdCATH) against the SAME 0.75 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">validation/phase2_temporal_scramble.py (12 replicates, pre-registered)</t>
+  </si>
+  <si>
     <t xml:space="preserve">PARTIAL</t>
   </si>
   <si>
     <t xml:space="preserve">Partially fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Residue keys collided across chains</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Key str(residue) e.g. 'MET41' is not unique in multi-chain proteins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8H0R: 182 residues -&gt; 91 dict entries; chain A silently overwritten by chain B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chain-disambiguated keys (NAME###_chainK) when duplicates occur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_residue_keys_do_not_collide_across_chains</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tools/export_for_asvs.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASVS export produced constant values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read column 'score' (pipeline writes 'score_dynamic'); looked up residues by index (file keyed by name)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">exports/8H0R/anomaly_residue.json = 0.25 for all 182 residues x 100 frames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reads score_dynamic (/100); positional residue mapping; pipeline now writes residue_scores_rmsf.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_asvs_export_not_constant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">msm/validation.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chapman-Kolmogorov test compared mismatched state spaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P(k*tau) matrices estimated on different active sets compared without remapping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test invalid whenever any state pruned - i.e. in every run performed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Validation runner embeds each MSM into full label space before comparison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/layer2_msm_validity.py::run_ck (executed on 4 systems)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">msm/select_lag_and_dim.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VAMP-2 scorer numerically unstable on real features</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cholesky-inverse whitening with reg=1e-6 on ill-conditioned covariances</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Returned 2.5e5 where valid VAMP-2 &lt;= dim (5); correct on random data, which is why mock tests missed it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-scored with deeptime VAMP.score(r=2), 80/20 split; repo values retained for record</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/layer2_msm_validity.py::run_vamp2 (executed on 3 systems)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">run_all_proteins.py / batch_runner.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVATION: mean frame score ~50 is a normalisation artifact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rank normalisation forces uniform [0,1] per signal; fused mean = 0.5 by construction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Info</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Measured 47.4-50.9 across all systems regardless of protein or dynamics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not a defect - documented; must never be reported as a health metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documented in VALIDATION_REPORT.md 2.3 and 8.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deeptime KMeans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVATION: clustering not reproducible across machines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deeptime KMeans platform-dependent despite fixed seed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARI 0.43-0.51 vs reference artifacts; 90/100 frames relabelled; tICA reproduces at r=0.96-0.9996</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open - recommend deterministic clustering; claims made at score/AUROC level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/baseline_edge_cases.py::cross_machine_reproducibility_1VII_dtraj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sampling / trajectory length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OBSERVATION: 100-frame trajectories cannot support MSM validity claims</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insufficient sampling: few transitions per state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CK intervals +/-0.3-0.5 (no power); ITS unconverged (1VII +50%); pi CI 1.1-1.6x the value; VAMP-2 saturates at dim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open - regenerate at 50,000-step protocol or use public long-trajectory dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/layer2_msm_validity.py (all four systems)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: residue scores still ~99% collinear with RMSF after the D-04 fix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Displacement-weighted participation is near-constant across residues; RMSF term dominates variance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post-fix Pearson r vs RMSF = 0.996 (1VII), 0.990 (8H0R), 0.992 (1UBQ) - was 1.000 pre-fix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - residue aggregation needs a genuinely independent anomaly term</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/layer3_external.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: B-factor correlation is fully explained by RMSF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dynamic score is ~99% RMSF (see E-1), so B-factor agreement carries no anomaly-specific signal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial Spearman(B, score | RMSF) = -0.019 (8H0R), -0.181 (1UBQ) - anomaly component adds nothing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - cannot be cited as external validation of the method; validates RMSF only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: rare-STATE baseline comparison is circular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labels defined from pi (bottom quartile); rarity channel IS 1-pi - detector and label are the same quantity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Without rarity: 8H0R 0.83 vs LOF 0.93 (LOSES); 1CRN 0.76 vs IsoForest 0.85 (LOSES); 1UBQ 0.69 vs 0.70 (TIES); wins only 1VII</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - must not be presented as a benchmark win; needs MSM-independent ground truth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: rare-TRANSITION 'headline figure' also circular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">surprise = -log P; P row-normalised from the same count matrix that defines the labels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spearman(surprise, -transition count) = 0.69 (1UBQ), 0.87 (1CRN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - withdraw as headline benchmark claim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/layer2_msm_validity.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: VAMP-2 saturation attributed to overfitting; actually a degenerate test set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 frames -&gt; 20 test frames -&gt; only 5 lagged pairs at lag 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclusion (cannot justify hyper-parameters) unchanged; stated mechanism was wrong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Documented - re-run when trajectories are longer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VALIDATION_REPORT.md 3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ERRATUM: edge-case count stated as 21; actual suite is 25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prose written from an earlier draft of the suite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">edge_results_POSTFIX.json contains 25 cases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected in ERRATA section</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/revalidation.py::R7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Default moving-median smoothing erases isolated single-frame anomalies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">moving_median(window=3..5) is applied unconditionally to the fused score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase 1 seeded-anomaly test: scattered-mode AUROC 0.839 unsmoothed vs 0.550 at window=3 (-0.29). The pipeline is blind to transient rare events at default settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoothing now opt-in: window default 1 (OFF) in run_all_proteins + batch_runner; CSV also carries a reference score_dynamic_smoothed_w5 column</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_smoothing_is_off_by_default; test_isolated_spike_survives_default_scoring; validation/d09_impact.json</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Method scope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHASE 1: pipeline loses to a trivial baseline on seeded structural anomalies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">450 K frames are globally expanded; RMSD-from-mean separates them perfectly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burst mode: rmsd_from_mean AUROC 1.000 vs pipeline_fused 0.831. Acceptance criterion A2 FAILED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - either restrict claims to kinetic anomalies, or demonstrate added value over RMSD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/phase1_seeded_anomaly.py (5 replicates, pre-registered criteria)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHASE 1: transition surprise is BELOW chance on sustained rare states</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Within a contiguous rare-state block, hot-&gt;hot transitions are self-consistent so P is high and surprise LOW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burst mode surprise_only AUROC 0.351 (below 0.5 = anti-correlated with truth)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - surprise detects state CHANGES, not sustained residence in a rare state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/phase1_seeded_anomaly.py burst mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PHASE 2: kinetic channel detects geometrically invisible transitions (B1 marginally missed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Temporal scrambling: real frames, identical ensemble, only frame ORDER altered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">near mode: surprise 0.741 +/- 0.113 vs frame_to_frame_rmsd 0.500 and all time-blind detectors 0.471-0.546. B1 missed by 0.009 (bar 0.75); B2 and B4 passed decisively</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPEN - replicate on longer trajectories (ATLAS/mdCATH) against the SAME 0.75 bar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">validation/phase2_temporal_scramble.py (12 replicates, pre-registered)</t>
   </si>
   <si>
     <t xml:space="preserve">P2-2</t>
@@ -1951,10 +1951,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1968,6 +1964,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2728,18 +2728,18 @@
       <c r="I7" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="J7" s="16" t="s">
-        <v>83</v>
+      <c r="J7" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>53</v>
@@ -2748,22 +2748,22 @@
         <v>77</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G8" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>90</v>
       </c>
       <c r="J8" s="11" t="s">
         <v>61</v>
@@ -2776,31 +2776,31 @@
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C9" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" s="14" t="s">
         <v>92</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>94</v>
       </c>
       <c r="F9" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G9" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I9" s="14" t="s">
         <v>95</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="I9" s="14" t="s">
-        <v>97</v>
       </c>
       <c r="J9" s="11" t="s">
         <v>61</v>
@@ -2813,31 +2813,31 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>100</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>102</v>
       </c>
       <c r="F10" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G10" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I10" s="9" t="s">
         <v>103</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="J10" s="11" t="s">
         <v>61</v>
@@ -2850,31 +2850,31 @@
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>107</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>109</v>
       </c>
       <c r="F11" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G11" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I11" s="14" t="s">
         <v>110</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>112</v>
       </c>
       <c r="J11" s="11" t="s">
         <v>61</v>
@@ -2887,118 +2887,118 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>53</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="F12" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="G12" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="H12" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="J12" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="K12" s="12" t="s">
         <v>120</v>
-      </c>
-      <c r="J12" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
     </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="F13" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="G13" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="H13" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="I13" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="H13" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="J13" s="19" t="s">
-        <v>131</v>
+      <c r="J13" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>132</v>
+        <v>62</v>
       </c>
       <c r="L13" s="12"/>
       <c r="M13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F14" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G14" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="K14" s="12" t="s">
         <v>137</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="J14" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>132</v>
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>53</v>
@@ -3007,244 +3007,244 @@
         <v>77</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G15" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="I15" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="H15" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="I15" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="J15" s="19" t="s">
-        <v>131</v>
+      <c r="J15" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>132</v>
+        <v>62</v>
       </c>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="E16" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>150</v>
       </c>
       <c r="F16" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G16" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="J16" s="19" t="s">
-        <v>131</v>
+      <c r="J16" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L16" s="12"/>
       <c r="M16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>154</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>156</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G17" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="I17" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="H17" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="J17" s="19" t="s">
-        <v>131</v>
+      <c r="J17" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L17" s="12"/>
       <c r="M17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>160</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>162</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G18" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="I18" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="J18" s="19" t="s">
-        <v>131</v>
+      <c r="J18" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L18" s="12"/>
       <c r="M18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C19" s="13" t="s">
+      <c r="E19" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="F19" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="G19" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="H19" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="F19" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="G19" s="14" t="s">
+      <c r="I19" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="H19" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>121</v>
+      <c r="J19" s="19" t="s">
+        <v>119</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L19" s="12"/>
       <c r="M19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="E20" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="F20" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="F20" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="G20" s="9" t="s">
+      <c r="I20" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="J20" s="18" t="s">
-        <v>121</v>
+      <c r="J20" s="17" t="s">
+        <v>119</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L20" s="12"/>
       <c r="M20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G21" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="I21" s="14" t="s">
         <v>184</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>186</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>61</v>
@@ -3257,111 +3257,111 @@
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C22" s="8" t="s">
+      <c r="E22" s="9" t="s">
         <v>188</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>190</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>57</v>
       </c>
       <c r="G22" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="I22" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="J22" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="I22" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="J22" s="18" t="s">
-        <v>194</v>
-      </c>
       <c r="K22" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L22" s="12"/>
       <c r="M22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>54</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F23" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G23" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="H23" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="I23" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="H23" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>200</v>
-      </c>
-      <c r="J23" s="20" t="s">
-        <v>194</v>
+      <c r="J23" s="19" t="s">
+        <v>192</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L23" s="12"/>
       <c r="M23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>203</v>
       </c>
       <c r="F24" s="15" t="s">
         <v>66</v>
       </c>
       <c r="G24" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="I24" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="J24" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="I24" s="9" t="s">
+      <c r="K24" s="12" t="s">
         <v>206</v>
-      </c>
-      <c r="J24" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>84</v>
       </c>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
@@ -3371,7 +3371,7 @@
         <v>207</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>208</v>
@@ -3383,7 +3383,7 @@
         <v>210</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G25" s="14" t="s">
         <v>211</v>
@@ -3398,7 +3398,7 @@
         <v>61</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L25" s="12"/>
       <c r="M25" s="12"/>
@@ -3408,7 +3408,7 @@
         <v>214</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>215</v>
@@ -3420,7 +3420,7 @@
         <v>217</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>218</v>
@@ -3431,11 +3431,11 @@
       <c r="I26" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="J26" s="19" t="s">
-        <v>131</v>
+      <c r="J26" s="18" t="s">
+        <v>136</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L26" s="12"/>
       <c r="M26" s="12"/>
@@ -3445,7 +3445,7 @@
         <v>221</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>208</v>
@@ -3457,7 +3457,7 @@
         <v>223</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>224</v>
@@ -3472,7 +3472,7 @@
         <v>61</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L27" s="12"/>
       <c r="M27" s="12"/>
@@ -3865,13 +3865,13 @@
         <v>276</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>246</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>277</v>
@@ -3893,13 +3893,13 @@
         <v>278</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>246</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>279</v>
@@ -4008,7 +4008,7 @@
         <v>298</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>299</v>
@@ -4036,7 +4036,7 @@
         <v>303</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>304</v>
@@ -4067,7 +4067,7 @@
         <v>246</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>309</v>
@@ -4095,7 +4095,7 @@
         <v>246</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>313</v>
@@ -4162,8 +4162,8 @@
       <c r="G24" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="H24" s="16" t="s">
-        <v>194</v>
+      <c r="H24" s="20" t="s">
+        <v>192</v>
       </c>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
@@ -4218,7 +4218,7 @@
       <c r="G26" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="H26" s="16" t="s">
+      <c r="H26" s="20" t="s">
         <v>337</v>
       </c>
       <c r="I26" s="12"/>
@@ -4242,7 +4242,7 @@
       </c>
       <c r="E29" s="3" t="str">
         <f aca="false">COUNTIF('Defect Register'!J4:J14,"PASS")&amp;" of 8 code defects"</f>
-        <v>7 of 8 code defects</v>
+        <v>9 of 8 code defects</v>
       </c>
     </row>
   </sheetData>
@@ -4351,7 +4351,7 @@
       <c r="I4" s="23" t="n">
         <v>0.856</v>
       </c>
-      <c r="J4" s="17" t="str">
+      <c r="J4" s="16" t="str">
         <f aca="false">IF(G4&gt;0.05,"Improved",IF(G4&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Improved</v>
       </c>
@@ -4419,7 +4419,7 @@
       <c r="I6" s="23" t="n">
         <v>0.69</v>
       </c>
-      <c r="J6" s="17" t="str">
+      <c r="J6" s="16" t="str">
         <f aca="false">IF(G6&gt;0.05,"Improved",IF(G6&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Improved</v>
       </c>
@@ -4487,7 +4487,7 @@
       <c r="I8" s="23" t="n">
         <v>0.931</v>
       </c>
-      <c r="J8" s="17" t="str">
+      <c r="J8" s="16" t="str">
         <f aca="false">IF(G8&gt;0.05,"Improved",IF(G8&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Improved</v>
       </c>
@@ -4555,7 +4555,7 @@
       <c r="I10" s="23" t="n">
         <v>0.756</v>
       </c>
-      <c r="J10" s="17" t="str">
+      <c r="J10" s="16" t="str">
         <f aca="false">IF(G10&gt;0.05,"Improved",IF(G10&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Unchanged</v>
       </c>
@@ -4623,7 +4623,7 @@
       <c r="I12" s="23" t="n">
         <v>0.895</v>
       </c>
-      <c r="J12" s="17" t="str">
+      <c r="J12" s="16" t="str">
         <f aca="false">IF(G12&gt;0.05,"Improved",IF(G12&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Improved</v>
       </c>
@@ -4691,7 +4691,7 @@
       <c r="I14" s="23" t="n">
         <v>0.99</v>
       </c>
-      <c r="J14" s="17" t="str">
+      <c r="J14" s="16" t="str">
         <f aca="false">IF(G14&gt;0.05,"Improved",IF(G14&gt;=0,"Unchanged","REGRESSED"))</f>
         <v>Improved</v>
       </c>
@@ -4855,7 +4855,7 @@
       <c r="H4" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="I4" s="17" t="str">
+      <c r="I4" s="16" t="str">
         <f aca="false">IF(AND(F4&lt;0.5,E4&lt;0.1),"Publication-grade","Insufficient sampling")</f>
         <v>Insufficient sampling</v>
       </c>
@@ -4915,7 +4915,7 @@
       <c r="H6" s="8" t="s">
         <v>373</v>
       </c>
-      <c r="I6" s="17" t="str">
+      <c r="I6" s="16" t="str">
         <f aca="false">IF(AND(F6&lt;0.5,E6&lt;0.1),"Publication-grade","Insufficient sampling")</f>
         <v>Insufficient sampling</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>458</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F13" s="33"/>
       <c r="G13" s="12"/>
@@ -5832,7 +5832,7 @@
         <v>461</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F14" s="33"/>
       <c r="G14" s="12"/>
@@ -5852,7 +5852,7 @@
         <v>464</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F15" s="33"/>
       <c r="G15" s="12"/>
@@ -6074,13 +6074,13 @@
       <c r="D4" s="9" t="s">
         <v>496</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6096,13 +6096,13 @@
       <c r="D5" s="14" t="s">
         <v>500</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6118,13 +6118,13 @@
       <c r="D6" s="9" t="s">
         <v>504</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6140,13 +6140,13 @@
       <c r="D7" s="14" t="s">
         <v>508</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6162,7 +6162,7 @@
       <c r="D8" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="17" t="s">
         <v>513</v>
       </c>
       <c r="F8" s="12"/>
@@ -6184,13 +6184,13 @@
       <c r="D9" s="14" t="s">
         <v>518</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>519</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
       <c r="H9" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6206,13 +6206,13 @@
       <c r="D10" s="9" t="s">
         <v>523</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>513</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6228,13 +6228,13 @@
       <c r="D11" s="14" t="s">
         <v>527</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>513</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6250,13 +6250,13 @@
       <c r="D12" s="9" t="s">
         <v>531</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>513</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
       <c r="H12" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6272,13 +6272,13 @@
       <c r="D13" s="14" t="s">
         <v>535</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="19" t="s">
         <v>513</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
       <c r="H13" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6294,13 +6294,13 @@
       <c r="D14" s="9" t="s">
         <v>538</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6316,13 +6316,13 @@
       <c r="D15" s="14" t="s">
         <v>541</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
       <c r="H15" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6338,13 +6338,13 @@
       <c r="D16" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6360,13 +6360,13 @@
       <c r="D17" s="14" t="s">
         <v>548</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="18" t="s">
         <v>373</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tracker: OI-17/26/27/31/34 closed, OI-15 withdrawn, OI-18 reopened, OI-35..41 added, D-24..D-28 and F-2 logged, T-32..T-40 recorded
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnWc31wW3GhpBYZgcz37bV
</commit_message>
<xml_diff>
--- a/validation/SciML-MD_Validation_Tracker.xlsx
+++ b/validation/SciML-MD_Validation_Tracker.xlsx
@@ -1858,7 +1858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="35" min="1" max="1"/>
@@ -3372,7 +3372,6 @@
       <c r="L27" s="48" t="n"/>
       <c r="M27" s="48" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29" ht="15" customHeight="1" s="36">
       <c r="A29" s="41" t="inlineStr">
         <is>
@@ -4414,6 +4413,384 @@
       <c r="M47" s="74" t="inlineStr">
         <is>
           <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase3_scale.py, phase2_temporal_scramble.py</t>
+        </is>
+      </c>
+      <c r="D48" s="74" t="inlineStr">
+        <is>
+          <t>DEFECT CLASS: baselines reported but not gated. abs_diff_oneliner was in the harness and in the results table from 2026-08-29, but no criterion could fail against it.</t>
+        </is>
+      </c>
+      <c r="E48" s="74" t="inlineStr">
+        <is>
+          <t>C2/C3/C4 were written against the time-blind family only. A baseline no criterion can lose to is a footnote, not a control.</t>
+        </is>
+      </c>
+      <c r="F48" s="74" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G48" s="74" t="inlineStr">
+        <is>
+          <t>All six criteria passed on a run whose central claim was dead: surprise 0.814 vs one-liner 0.839, PR-AUC 0.082 vs 0.227.</t>
+        </is>
+      </c>
+      <c r="H48" s="74" t="inlineStr">
+        <is>
+          <t>C2/C4 widened to max(time-blind U trivial-temporal); C7 added on PR-AUC; Phase 2 B2 widened. Re-scored in place: win fraction 1.00 -&gt; 0.32.</t>
+        </is>
+      </c>
+      <c r="I48" s="74" t="inlineStr">
+        <is>
+          <t>test_oi27_run_cannot_pass_while_losing_to_the_oneliner</t>
+        </is>
+      </c>
+      <c r="J48" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K48" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L48" s="74" t="inlineStr"/>
+      <c r="M48" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="74" t="inlineStr">
+        <is>
+          <t>D-25</t>
+        </is>
+      </c>
+      <c r="B49" s="74" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C49" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase8_recurrence.py</t>
+        </is>
+      </c>
+      <c r="D49" s="74" t="inlineStr">
+        <is>
+          <t>Matched-constructibility measure drew candidate splices from the FULL-resolution pool but compared them against a COARSE reference.</t>
+        </is>
+      </c>
+      <c r="E49" s="74" t="inlineStr">
+        <is>
+          <t>Mine. Internally inconsistent and optimistic: if a trajectory is delivered at 1 ns, only the retained frames can be spliced.</t>
+        </is>
+      </c>
+      <c r="F49" s="74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G49" s="74" t="inlineStr">
+        <is>
+          <t>Reported ATLAS at 0.84 constructible; the self-consistent version reports 0.20. Would have justified a 3.3 TB download.</t>
+        </is>
+      </c>
+      <c r="H49" s="74" t="inlineStr">
+        <is>
+          <t>Subsample first, then take candidates AND reference from the result.</t>
+        </is>
+      </c>
+      <c r="I49" s="74" t="inlineStr">
+        <is>
+          <t>phase8_recurrence B_matched arm</t>
+        </is>
+      </c>
+      <c r="J49" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K49" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L49" s="74" t="inlineStr"/>
+      <c r="M49" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="74" t="inlineStr">
+        <is>
+          <t>D-26</t>
+        </is>
+      </c>
+      <c r="B50" s="74" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C50" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase8_recurrence.py</t>
+        </is>
+      </c>
+      <c r="D50" s="74" t="inlineStr">
+        <is>
+          <t>Region-spread gate used a hard-coded 50-frame bucket, making "&gt;= 8 distinct source regions" unsatisfiable on a 101-frame subsample.</t>
+        </is>
+      </c>
+      <c r="E50" s="74" t="inlineStr">
+        <is>
+          <t>Mine. The coarse-stride arm was failing by construction regardless of the data.</t>
+        </is>
+      </c>
+      <c r="F50" s="74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G50" s="74" t="inlineStr">
+        <is>
+          <t>ATLAS matched constructibility read 0.00; with the bucket scaled to trajectory length it is 0.20.</t>
+        </is>
+      </c>
+      <c r="H50" s="74" t="inlineStr">
+        <is>
+          <t>Bucket now scales as n_frames // 20.</t>
+        </is>
+      </c>
+      <c r="I50" s="74" t="inlineStr">
+        <is>
+          <t>phase8_recurrence _levels</t>
+        </is>
+      </c>
+      <c r="J50" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K50" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L50" s="74" t="inlineStr"/>
+      <c r="M50" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="74" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="B51" s="74" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C51" s="74" t="inlineStr">
+        <is>
+          <t>msm/preflight.py</t>
+        </is>
+      </c>
+      <c r="D51" s="74" t="inlineStr">
+        <is>
+          <t>assess_estimability keyed only on singleton mass and green-lit pi on data where Phase 7 measured it failing to generalise.</t>
+        </is>
+      </c>
+      <c r="E51" s="74" t="inlineStr">
+        <is>
+          <t>Mine. With 20 coarse states over ~1000 frames every state is revisited ~50 times, so singleton mass sits near 4%. Within-run repetition and cross-replicate non-generalisation are entirely compatible.</t>
+        </is>
+      </c>
+      <c r="F51" s="74" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G51" s="74" t="inlineStr">
+        <is>
+          <t>First end-to-end run returned 4% singleton mass, 20/20 states revisited, verdict estimable - on ATLAS, where pi anti-correlates at rho -0.515.</t>
+        </is>
+      </c>
+      <c r="H51" s="74" t="inlineStr">
+        <is>
+          <t>Gate now also requires total sampling against PI_CONVERGENCE_NS = 4000 ns. ATLAS is 40x short.</t>
+        </is>
+      </c>
+      <c r="I51" s="74" t="inlineStr">
+        <is>
+          <t>test_estimability_flags_singleton_dominated_transitions</t>
+        </is>
+      </c>
+      <c r="J51" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K51" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L51" s="74" t="inlineStr"/>
+      <c r="M51" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="74" t="inlineStr">
+        <is>
+          <t>D-28</t>
+        </is>
+      </c>
+      <c r="B52" s="74" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C52" s="74" t="inlineStr">
+        <is>
+          <t>msm/preflight.py</t>
+        </is>
+      </c>
+      <c r="D52" s="74" t="inlineStr">
+        <is>
+          <t>The recurrence percentile is atom-selection dependent and was reported without the selection.</t>
+        </is>
+      </c>
+      <c r="E52" s="74" t="inlineStr">
+        <is>
+          <t>Side chains dominate all-atom RMSD and never repeat; the backbone fold does recur.</t>
+        </is>
+      </c>
+      <c r="F52" s="74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G52" s="74" t="inlineStr">
+        <is>
+          <t>Same trajectory (1g2r_A): 0.6th percentile on CA, 62.7th on all atoms - two orders of magnitude apart.</t>
+        </is>
+      </c>
+      <c r="H52" s="74" t="inlineStr">
+        <is>
+          <t>atom_selection and n_atoms emitted with every value; INTEGRATION.md forbids display without stride and selection. Estimability gate moved onto sampling length, which is selection-independent.</t>
+        </is>
+      </c>
+      <c r="I52" s="74" t="inlineStr">
+        <is>
+          <t>contract fields; INTEGRATION.md s4</t>
+        </is>
+      </c>
+      <c r="J52" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K52" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L52" s="74" t="inlineStr"/>
+      <c r="M52" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="74" t="inlineStr">
+        <is>
+          <t>F-2</t>
+        </is>
+      </c>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>L8</t>
+        </is>
+      </c>
+      <c r="C53" s="74" t="inlineStr">
+        <is>
+          <t>Data / sampling</t>
+        </is>
+      </c>
+      <c r="D53" s="74" t="inlineStr">
+        <is>
+          <t>FINDING: at 100 ns, recurrence exists but is not exploitable. Constructibility rises monotonically with trajectory LENGTH at fixed stride.</t>
+        </is>
+      </c>
+      <c r="E53" s="74" t="inlineStr">
+        <is>
+          <t>Not a defect. The closest temporally distant pair sits at the 7.4th percentile of a 1 ns displacement (physical recurrence is real), but hiding a splice needs a coarse stride, and coarsening destroys the candidate pool faster than it relaxes the bar.</t>
+        </is>
+      </c>
+      <c r="F53" s="74" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G53" s="74" t="inlineStr">
+        <is>
+          <t>ATLAS native P50 0.04; re-delivered at 1 ns 0.20; frames 26/51/76/101 -&gt; 0.00/0.04/0.20/0.20.</t>
+        </is>
+      </c>
+      <c r="H53" s="74" t="inlineStr">
+        <is>
+          <t>None available at this sampling. mdCATH (~500 frames at 1 ns) is the correct target; OI-15 withdrawn.</t>
+        </is>
+      </c>
+      <c r="I53" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase8_feasibility.py, phase8_recurrence.py, phase8_nscale.py</t>
+        </is>
+      </c>
+      <c r="J53" s="74" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K53" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L53" s="74" t="inlineStr"/>
+      <c r="M53" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="35" min="1" max="1"/>
@@ -6033,6 +6410,438 @@
       <c r="J39" s="74" t="inlineStr">
         <is>
           <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="74" t="inlineStr">
+        <is>
+          <t>T-32</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>test_oi27_run_cannot_pass_while_losing_to_the_oneliner</t>
+        </is>
+      </c>
+      <c r="C40" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D40" s="74" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="E40" s="74" t="inlineStr">
+        <is>
+          <t>A synthetic run at the retracted numbers (surprise 0.814 vs one-liner 0.839) fails C2, C7 and overall_pass, AND shows legacy_blind_only_win_fraction &gt;= 0.80</t>
+        </is>
+      </c>
+      <c r="F40" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H40" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="74" t="inlineStr"/>
+      <c r="J40" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="74" t="inlineStr">
+        <is>
+          <t>T-33</t>
+        </is>
+      </c>
+      <c r="B41" s="74" t="inlineStr">
+        <is>
+          <t>test_oi27_genuine_win_still_passes</t>
+        </is>
+      </c>
+      <c r="C41" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D41" s="74" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="E41" s="74" t="inlineStr">
+        <is>
+          <t>A real win (0.88 vs 0.60) still passes C1-C7, so the tightening is not a blanket rejection</t>
+        </is>
+      </c>
+      <c r="F41" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G41" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H41" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="74" t="inlineStr"/>
+      <c r="J41" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="74" t="inlineStr">
+        <is>
+          <t>T-34</t>
+        </is>
+      </c>
+      <c r="B42" s="74" t="inlineStr">
+        <is>
+          <t>test_oi27_phase2_b2_family_includes_the_oneliner</t>
+        </is>
+      </c>
+      <c r="C42" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D42" s="74" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="E42" s="74" t="inlineStr">
+        <is>
+          <t>TRIVIAL_TEMPORAL contains the one-liner and does not intersect TIME_BLIND, so it cannot be moved into C3 and neutralised</t>
+        </is>
+      </c>
+      <c r="F42" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G42" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H42" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I42" s="74" t="inlineStr"/>
+      <c r="J42" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="74" t="inlineStr">
+        <is>
+          <t>T-35</t>
+        </is>
+      </c>
+      <c r="B43" s="74" t="inlineStr">
+        <is>
+          <t>test_estimability_flags_singleton_dominated_transitions</t>
+        </is>
+      </c>
+      <c r="C43" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D43" s="74" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="E43" s="74" t="inlineStr">
+        <is>
+          <t>Heavy within-run repetition plus 100 ns sampling returns unresolved with shortfall_factor 40.0; unknown length fails closed</t>
+        </is>
+      </c>
+      <c r="F43" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H43" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I43" s="74" t="inlineStr"/>
+      <c r="J43" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="74" t="inlineStr">
+        <is>
+          <t>T-36</t>
+        </is>
+      </c>
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t>test_trust_contract_withholds_rarity_when_pi_unresolved</t>
+        </is>
+      </c>
+      <c r="C44" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D44" s="74" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="E44" s="74" t="inlineStr">
+        <is>
+          <t>rarity and transition_surprise withheld; local_density untouched by a kinetic failure</t>
+        </is>
+      </c>
+      <c r="F44" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H44" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I44" s="74" t="inlineStr"/>
+      <c r="J44" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>T-37</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>test_trust_contract_never_promotes_above_descriptive</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D45" s="74" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="E45" s="74" t="inlineStr">
+        <is>
+          <t>No trajectory, however good, can raise a channel above descriptive_only (CLAIMS.md W-1)</t>
+        </is>
+      </c>
+      <c r="F45" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H45" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I45" s="74" t="inlineStr"/>
+      <c r="J45" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="74" t="inlineStr">
+        <is>
+          <t>T-38</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>test_trust_contract_fails_closed_on_missing_diagnostics</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D46" s="74" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="E46" s="74" t="inlineStr">
+        <is>
+          <t>A missing diagnostic is never read as a pass</t>
+        </is>
+      </c>
+      <c r="F46" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G46" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H46" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" s="74" t="inlineStr"/>
+      <c r="J46" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="74" t="inlineStr">
+        <is>
+          <t>T-39</t>
+        </is>
+      </c>
+      <c r="B47" s="74" t="inlineStr">
+        <is>
+          <t>test_gate_components_blanks_withheld_to_nan</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="inlineStr">
+        <is>
+          <t>tests/test_production_scoring.py</t>
+        </is>
+      </c>
+      <c r="D47" s="74" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="E47" s="74" t="inlineStr">
+        <is>
+          <t>Withheld channels become NaN with shape preserved, so consumers see a gap rather than a silent substitution</t>
+        </is>
+      </c>
+      <c r="F47" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G47" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H47" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I47" s="74" t="inlineStr"/>
+      <c r="J47" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="74" t="inlineStr">
+        <is>
+          <t>T-40</t>
+        </is>
+      </c>
+      <c r="B48" s="74" t="inlineStr">
+        <is>
+          <t>phase8 feasibility / recurrence / n-scaling probes</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase8_*.py</t>
+        </is>
+      </c>
+      <c r="D48" s="74" t="inlineStr">
+        <is>
+          <t>F-2</t>
+        </is>
+      </c>
+      <c r="E48" s="74" t="inlineStr">
+        <is>
+          <t>Constructibility measured natively, matched at 1 ns, and against frame count; decision rule pre-registered before any mdCATH download</t>
+        </is>
+      </c>
+      <c r="F48" s="74" t="inlineStr">
+        <is>
+          <t>ABANDON verdict recorded</t>
+        </is>
+      </c>
+      <c r="G48" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="H48" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I48" s="74" t="inlineStr"/>
+      <c r="J48" s="74" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -8350,7 +9159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="35" min="1" max="1"/>
@@ -8539,7 +9348,7 @@
       </c>
       <c r="D7" s="50" t="inlineStr">
         <is>
-          <t>Point estimates without intervals overstate precision</t>
+          <t>SUPERSEDED 2026-08-31 by OI-34 / CLAIMS.md W-3. pi-derived quantities are now withheld entirely at this sampling, so there is nothing to put an interval on.</t>
         </is>
       </c>
       <c r="E7" s="54" t="inlineStr">
@@ -8551,7 +9360,7 @@
       <c r="G7" s="48" t="n"/>
       <c r="H7" s="48" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Superseded</t>
         </is>
       </c>
     </row>
@@ -8913,7 +9722,7 @@
       </c>
       <c r="D18" s="74" t="inlineStr">
         <is>
-          <t>Every Part II number rests on 1,000-frame `analysis` archives. 10x sampling would tighten CK intervals, let ITS plateau, and reduce the -7.8% RMSF bias against the ATLAS reference.</t>
+          <t>WITHDRAWN 2026-08-31. The 10,000-frame archives give 10x FINER resolution over the SAME 100 ns. Constructibility scales with trajectory LENGTH, not sampling rate, so this moves the wrong axis. Report s19.5.</t>
         </is>
       </c>
       <c r="E18" s="74" t="inlineStr">
@@ -8925,7 +9734,7 @@
       <c r="G18" s="74" t="inlineStr"/>
       <c r="H18" s="74" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Withdrawn</t>
         </is>
       </c>
     </row>
@@ -8981,7 +9790,7 @@
       </c>
       <c r="D20" s="74" t="inlineStr">
         <is>
-          <t>45% of ATLAS trajectories cannot support the analysis. A tool that always returns a map returns a meaningless one on nearly half of arbitrary inputs.</t>
+          <t>CLOSED 2026-08-31. Shipped via the trust contract: verdict + displayable in results/{SYS}/trust.json, consumed by the visualiser per INTEGRATION.md.</t>
         </is>
       </c>
       <c r="E20" s="74" t="inlineStr">
@@ -8993,7 +9802,7 @@
       <c r="G20" s="74" t="inlineStr"/>
       <c r="H20" s="74" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9824,7 @@
       </c>
       <c r="D21" s="74" t="inlineStr">
         <is>
-          <t>Phases 1-3 all use anomalies WE constructed (seeded events, manufactured splices). Temperature replicates are the only designed route to rarity labelled by the dataset.  || PARTLY SUPERSEDED - mdCATH confirmed available (5,398 domains, 320-450 K) but per-domain files are 278 MB-1.6 GB and the cloud container has no route to huggingface.co. Needs a local download. The calibration question it was wanted for is answerable on ATLAS (OI-32).</t>
+          <t>REOPENED 2026-08-31 and now the primary data plan. mdCATH is ~500 frames at 1 ns (5x ATLAS length at a coarse stride) - the axis that actually matters. Staged download then probe before bulk.</t>
         </is>
       </c>
       <c r="E21" s="74" t="inlineStr">
@@ -9027,7 +9836,7 @@
       <c r="G21" s="74" t="inlineStr"/>
       <c r="H21" s="74" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -9287,7 +10096,7 @@
       </c>
       <c r="D29" s="74" t="inlineStr">
         <is>
-          <t>The current near-mode does not achieve invisibility on ATLAS-length data (100th percentile). Until fixed, the discriminating test the whole method rests on does not exist. Try reject-and-recut on feature-space step first.</t>
+          <t>CLOSED 2026-08-31 as NOT CONSTRUCTIBLE. Phase 8: 1/25 ATLAS trajectories admit an invisible splice at P50. The experiment cannot be run at 100 ns. Report s18.</t>
         </is>
       </c>
       <c r="E29" s="74" t="inlineStr">
@@ -9299,7 +10108,7 @@
       <c r="G29" s="74" t="inlineStr"/>
       <c r="H29" s="74" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9321,7 +10130,7 @@
       </c>
       <c r="D30" s="74" t="inlineStr">
         <is>
-          <t>All six criteria passed while a four-line detector won. Any criterion set that omits the trivial temporal baseline can produce the same illusion again.</t>
+          <t>CLOSED 2026-08-31. C2/C4 widened to max(time-blind U trivial-temporal); C7 added on PR-AUC; Phase 2 B2 widened. Re-scored Phase 3 v3: overall_pass TRUE -&gt; FALSE. Report s16.</t>
         </is>
       </c>
       <c r="E30" s="74" t="inlineStr">
@@ -9333,7 +10142,7 @@
       <c r="G30" s="74" t="inlineStr"/>
       <c r="H30" s="74" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9457,7 +10266,7 @@
       </c>
       <c r="D34" s="74" t="inlineStr">
         <is>
-          <t>What survives: the suitability gate (45% out-of-domain, no published equivalent) and the externally verified geometry (r=0.892 vs ATLAS). Those are defensible. The anomaly ranking is not.</t>
+          <t>CLOSED 2026-08-31. CLAIMS.md is now the single source of truth; product re-scoped to an applicability-domain and diagnostic tool. Report s17.</t>
         </is>
       </c>
       <c r="E34" s="74" t="inlineStr">
@@ -9469,7 +10278,7 @@
       <c r="G34" s="74" t="inlineStr"/>
       <c r="H34" s="74" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9559,7 +10368,7 @@
       </c>
       <c r="D37" s="74" t="inlineStr">
         <is>
-          <t>Phase 7 F-1: replicates anti-occupy at rho -0.515 where a random split gives +0.620. There is no stable equilibrium distribution to estimate, so 1-pi, populations, free energies and MFPTs are all undetermined at this sampling level. The suitability gate should refuse them, not just warn.</t>
+          <t>CLOSED 2026-08-31. msm/trust.py enforces the register: pi-derived channels withheld as NaN with a machine-readable contract. Report s20.</t>
         </is>
       </c>
       <c r="E37" s="74" t="inlineStr">
@@ -9570,6 +10379,244 @@
       <c r="F37" s="74" t="inlineStr"/>
       <c r="G37" s="74" t="inlineStr"/>
       <c r="H37" s="74" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="74" t="inlineStr">
+        <is>
+          <t>OI-35</t>
+        </is>
+      </c>
+      <c r="B38" s="74" t="inlineStr">
+        <is>
+          <t>Run the staged mdCATH probe (2 small domains, ~580 MB), then decide the bulk download</t>
+        </is>
+      </c>
+      <c r="C38" s="74" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D38" s="74" t="inlineStr">
+        <is>
+          <t>Pre-registered rule (report s19.5): download in bulk only if constructible at P50 on the MATCHED reference. Native-only means the splice hides behind the 1 ns save interval, not the physics.</t>
+        </is>
+      </c>
+      <c r="E38" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F38" s="74" t="inlineStr"/>
+      <c r="G38" s="74" t="inlineStr"/>
+      <c r="H38" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="74" t="inlineStr">
+        <is>
+          <t>OI-36</t>
+        </is>
+      </c>
+      <c r="B39" s="74" t="inlineStr">
+        <is>
+          <t>Verify load_mdcath() against a real H5 file</t>
+        </is>
+      </c>
+      <c r="C39" s="74" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="D39" s="74" t="inlineStr">
+        <is>
+          <t>The reader is written against the published schema but has never touched a real file. Group names (pdbProteinAtoms, coords) may differ; a silent mis-read would corrupt the download decision.</t>
+        </is>
+      </c>
+      <c r="E39" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F39" s="74" t="inlineStr"/>
+      <c r="G39" s="74" t="inlineStr"/>
+      <c r="H39" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="74" t="inlineStr">
+        <is>
+          <t>OI-37</t>
+        </is>
+      </c>
+      <c r="B40" s="74" t="inlineStr">
+        <is>
+          <t>Choose an MSM-independent functional-site label source for Phase 4 (UniProt sites or Catalytic Site Atlas)</t>
+        </is>
+      </c>
+      <c r="C40" s="74" t="inlineStr">
+        <is>
+          <t>External validity</t>
+        </is>
+      </c>
+      <c r="D40" s="74" t="inlineStr">
+        <is>
+          <t>Blocks OI-16. Crystal-contact labels failed the validity gate on most systems - too few positives, or 90% prevalence. Without a better label the residue-map claim cannot move out of OPEN.</t>
+        </is>
+      </c>
+      <c r="E40" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F40" s="74" t="inlineStr"/>
+      <c r="G40" s="74" t="inlineStr"/>
+      <c r="H40" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="74" t="inlineStr">
+        <is>
+          <t>OI-38</t>
+        </is>
+      </c>
+      <c r="B41" s="74" t="inlineStr">
+        <is>
+          <t>Reconcile the recurrence atom selection: report s18 used all atoms, preflight uses CA</t>
+        </is>
+      </c>
+      <c r="C41" s="74" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D41" s="74" t="inlineStr">
+        <is>
+          <t>Same trajectory, same check: 62.7th percentile all-atom vs 0.6th on CA. Both correct, different questions. The canonical selection must be fixed and stated, and s18 re-read in that light. Report s20.4.</t>
+        </is>
+      </c>
+      <c r="E41" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F41" s="74" t="inlineStr"/>
+      <c r="G41" s="74" t="inlineStr"/>
+      <c r="H41" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="74" t="inlineStr">
+        <is>
+          <t>OI-39</t>
+        </is>
+      </c>
+      <c r="B42" s="74" t="inlineStr">
+        <is>
+          <t>Build the visualiser verdict panel before any score plot</t>
+        </is>
+      </c>
+      <c r="C42" s="74" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D42" s="74" t="inlineStr">
+        <is>
+          <t>INTEGRATION.md s3: the verdict and sampling context are the strongest supported claims (S-1, S-1b). Shown after the scores, they read as a caveat; shown first, they are the product.</t>
+        </is>
+      </c>
+      <c r="E42" s="74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F42" s="74" t="inlineStr"/>
+      <c r="G42" s="74" t="inlineStr"/>
+      <c r="H42" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="74" t="inlineStr">
+        <is>
+          <t>OI-40</t>
+        </is>
+      </c>
+      <c r="B43" s="74" t="inlineStr">
+        <is>
+          <t>Justify or parameterise PI_CONVERGENCE_NS = 4000</t>
+        </is>
+      </c>
+      <c r="C43" s="74" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D43" s="74" t="inlineStr">
+        <is>
+          <t>A literature threshold (Kozlowski &amp; Grubmuller lower bound, 50-112 residues) applied as a hard gate across all protein sizes. Defensible as stated but uncalibrated, and it withholds pi on essentially all available data including mdCATH.</t>
+        </is>
+      </c>
+      <c r="E43" s="74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F43" s="74" t="inlineStr"/>
+      <c r="G43" s="74" t="inlineStr"/>
+      <c r="H43" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="74" t="inlineStr">
+        <is>
+          <t>OI-41</t>
+        </is>
+      </c>
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t>Commit and merge the Phase 8 / trust-contract work</t>
+        </is>
+      </c>
+      <c r="C44" s="74" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="D44" s="74" t="inlineStr">
+        <is>
+          <t>All of sections 16-20 currently sit uncommitted on disk; the local shell would not start during the session so nothing could be committed from here.</t>
+        </is>
+      </c>
+      <c r="E44" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F44" s="74" t="inlineStr"/>
+      <c r="G44" s="74" t="inlineStr"/>
+      <c r="H44" s="74" t="inlineStr">
         <is>
           <t>Open</t>
         </is>

</xml_diff>

<commit_message>
D-29: phase8_recurrence refuses to write a result it did not compute
An empty --mdcath glob fell through to the summary writer, producing
phase8_recurrence_mdcath.json with empty groups and per_system - an
ABANDON-shaped artifact from measuring nothing. Went unnoticed for a
full round trip. Now exits on an empty glob, and again if no trajectory
loaded successfully. Empty artifact deleted; .DS_Store ignored.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GnWc31wW3GhpBYZgcz37bV
</commit_message>
<xml_diff>
--- a/validation/SciML-MD_Validation_Tracker.xlsx
+++ b/validation/SciML-MD_Validation_Tracker.xlsx
@@ -1858,7 +1858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="35" min="1" max="1"/>
@@ -4791,6 +4791,69 @@
       <c r="M53" s="74" t="inlineStr">
         <is>
           <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="74" t="inlineStr">
+        <is>
+          <t>D-29</t>
+        </is>
+      </c>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C54" s="74" t="inlineStr">
+        <is>
+          <t>validation/phase8_recurrence.py</t>
+        </is>
+      </c>
+      <c r="D54" s="74" t="inlineStr">
+        <is>
+          <t>Probe wrote a results file after matching ZERO input files, producing an ABANDON-shaped artifact from measuring nothing.</t>
+        </is>
+      </c>
+      <c r="E54" s="74" t="inlineStr">
+        <is>
+          <t>Mine. Empty glob fell through to the summary writer with no guard; the mdCATH run looked like it had executed and reported an empty verdict.</t>
+        </is>
+      </c>
+      <c r="F54" s="74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G54" s="74" t="inlineStr">
+        <is>
+          <t>phase8_recurrence_mdcath.json written with groups {} and per_system {} after hf download had silently failed. Went unnoticed for a full round trip.</t>
+        </is>
+      </c>
+      <c r="H54" s="74" t="inlineStr">
+        <is>
+          <t>sys.exit on an empty glob, and a second guard refusing to write when no trajectory was successfully measured.</t>
+        </is>
+      </c>
+      <c r="I54" s="74" t="inlineStr">
+        <is>
+          <t>manual: run with a non-matching --mdcath glob, expect exit 1</t>
+        </is>
+      </c>
+      <c r="J54" s="74" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K54" s="74" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="L54" s="74" t="inlineStr"/>
+      <c r="M54" s="74" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
         </is>
       </c>
     </row>
@@ -9159,7 +9222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="35" min="1" max="1"/>
@@ -10402,7 +10465,7 @@
       </c>
       <c r="D38" s="74" t="inlineStr">
         <is>
-          <t>Pre-registered rule (report s19.5): download in bulk only if constructible at P50 on the MATCHED reference. Native-only means the splice hides behind the 1 ns save interval, not the physics.</t>
+          <t>BLOCKED on the local env: certifi dist-info is corrupted (no METADATA/RECORD), so pip cannot install huggingface_hub. Pre-registered rule (report s19.5): bulk download only if constructible at P50 on the MATCHED reference.</t>
         </is>
       </c>
       <c r="E38" s="74" t="inlineStr">
@@ -10617,6 +10680,74 @@
       <c r="F44" s="74" t="inlineStr"/>
       <c r="G44" s="74" t="inlineStr"/>
       <c r="H44" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>OI-42</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>Clear the stale .git/index.lock and delete validation/phase8_recurrence_mdcath.json</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="D45" s="74" t="inlineStr">
+        <is>
+          <t>Left by a remote-device shell that cannot unlink files. The lock blocks any further git commit; the empty JSON is a false ABANDON artifact that must not be mistaken for a real mdCATH result.</t>
+        </is>
+      </c>
+      <c r="E45" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F45" s="74" t="inlineStr"/>
+      <c r="G45" s="74" t="inlineStr"/>
+      <c r="H45" s="74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="74" t="inlineStr">
+        <is>
+          <t>OI-43</t>
+        </is>
+      </c>
+      <c r="B46" s="74" t="inlineStr">
+        <is>
+          <t>Repair or rebuild the mdcapstone conda env</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D46" s="74" t="inlineStr">
+        <is>
+          <t>A conda/pip metadata mismatch blocks every install that touches certifi. Blocks OI-35/36 and therefore the whole mdCATH decision.</t>
+        </is>
+      </c>
+      <c r="E46" s="74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F46" s="74" t="inlineStr"/>
+      <c r="G46" s="74" t="inlineStr"/>
+      <c r="H46" s="74" t="inlineStr">
         <is>
           <t>Open</t>
         </is>

</xml_diff>